<commit_message>
SE CAMBIARON LOS NOMBRES A MAYUSCULAS
</commit_message>
<xml_diff>
--- a/DOCUMENTOS FASE1/PLANILLA DE EVALUACIÓN FASE 1.xlsx
+++ b/DOCUMENTOS FASE1/PLANILLA DE EVALUACIÓN FASE 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SSDD\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C1BBC1-263E-42D6-8BAE-52D889742A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D19073F-846C-4CB4-99A1-B4EE1E99EA5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -383,16 +383,16 @@
     <t>Muy Relevante</t>
   </si>
   <si>
-    <t>Raúl Ignacio Ibarra Carvajal</t>
+    <t>RAUL IGNACIO IBARRA CARVAJAL</t>
   </si>
   <si>
-    <t>Javier Ignacio Perez Arenas</t>
+    <t>JAVIER IGNACIO PEREZ ARENAS</t>
   </si>
   <si>
-    <t>Jose Magdiel Gonzalez Lonconanco</t>
+    <t>JOSE MAGDIEL GONZALEZ LONCONANCO</t>
   </si>
   <si>
-    <t>Emanuel Eduardo Meza Burgos</t>
+    <t>EMANUEL EDUARDO MEZA BURGOS</t>
   </si>
 </sst>
 </file>
@@ -1059,6 +1059,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1067,18 +1070,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1580,22 +1580,22 @@
         <v>3</v>
       </c>
       <c r="B11" s="14"/>
-      <c r="C11" s="57" t="s">
+      <c r="C11" s="51" t="s">
         <v>4</v>
       </c>
       <c r="D11" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="59"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="59"/>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="60"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="62"/>
+      <c r="I11" s="62"/>
+      <c r="J11" s="62"/>
+      <c r="K11" s="59"/>
     </row>
     <row r="12" spans="1:11" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="62"/>
+      <c r="A12" s="61"/>
       <c r="B12" s="24" t="s">
         <v>6</v>
       </c>
@@ -1603,19 +1603,19 @@
       <c r="D12" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="60"/>
+      <c r="E12" s="59"/>
       <c r="F12" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="60"/>
+      <c r="G12" s="59"/>
       <c r="H12" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="I12" s="60"/>
+      <c r="I12" s="59"/>
       <c r="J12" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K12" s="60"/>
+      <c r="K12" s="59"/>
     </row>
     <row r="13" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A13" s="65"/>
@@ -2039,7 +2039,7 @@
       </c>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="62"/>
+      <c r="A23" s="61"/>
       <c r="B23" s="34" t="s">
         <v>11</v>
       </c>
@@ -2081,59 +2081,59 @@
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="61" t="s">
+      <c r="A27" s="60" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="51" t="str">
+      <c r="C27" s="52" t="str">
         <f>$B$4</f>
-        <v>Raúl Ignacio Ibarra Carvajal</v>
-      </c>
-      <c r="D27" s="52"/>
-      <c r="E27" s="52"/>
-      <c r="F27" s="52"/>
-      <c r="G27" s="52"/>
-      <c r="H27" s="52"/>
-      <c r="I27" s="52"/>
-      <c r="J27" s="52"/>
-      <c r="K27" s="53"/>
+        <v>RAUL IGNACIO IBARRA CARVAJAL</v>
+      </c>
+      <c r="D27" s="53"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="53"/>
+      <c r="G27" s="53"/>
+      <c r="H27" s="53"/>
+      <c r="I27" s="53"/>
+      <c r="J27" s="53"/>
+      <c r="K27" s="54"/>
     </row>
     <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="62"/>
+      <c r="A28" s="61"/>
       <c r="B28" s="50"/>
-      <c r="C28" s="54"/>
-      <c r="D28" s="55"/>
-      <c r="E28" s="55"/>
-      <c r="F28" s="55"/>
-      <c r="G28" s="55"/>
-      <c r="H28" s="55"/>
-      <c r="I28" s="55"/>
-      <c r="J28" s="55"/>
-      <c r="K28" s="56"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="56"/>
+      <c r="E28" s="56"/>
+      <c r="F28" s="56"/>
+      <c r="G28" s="56"/>
+      <c r="H28" s="56"/>
+      <c r="I28" s="56"/>
+      <c r="J28" s="56"/>
+      <c r="K28" s="57"/>
     </row>
     <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="62"/>
+      <c r="A29" s="61"/>
       <c r="B29" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="57" t="s">
+      <c r="C29" s="51" t="s">
         <v>4</v>
       </c>
       <c r="D29" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E29" s="59"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="59"/>
-      <c r="H29" s="59"/>
-      <c r="I29" s="59"/>
-      <c r="J29" s="59"/>
-      <c r="K29" s="60"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="62"/>
+      <c r="H29" s="62"/>
+      <c r="I29" s="62"/>
+      <c r="J29" s="62"/>
+      <c r="K29" s="59"/>
     </row>
     <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="62"/>
+      <c r="A30" s="61"/>
       <c r="B30" s="15" t="s">
         <v>6</v>
       </c>
@@ -2141,22 +2141,22 @@
       <c r="D30" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="60"/>
+      <c r="E30" s="59"/>
       <c r="F30" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G30" s="60"/>
+      <c r="G30" s="59"/>
       <c r="H30" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I30" s="60"/>
+      <c r="I30" s="59"/>
       <c r="J30" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K30" s="60"/>
+      <c r="K30" s="59"/>
     </row>
     <row r="31" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="62"/>
+      <c r="A31" s="61"/>
       <c r="B31" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2198,7 +2198,7 @@
       </c>
     </row>
     <row r="32" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="62"/>
+      <c r="A32" s="61"/>
       <c r="B32" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2240,7 +2240,7 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="62"/>
+      <c r="A33" s="61"/>
       <c r="B33" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2282,7 +2282,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="62"/>
+      <c r="A34" s="61"/>
       <c r="B34" s="21" t="s">
         <v>17</v>
       </c>
@@ -2331,59 +2331,59 @@
     </row>
     <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="61" t="s">
+      <c r="A39" s="60" t="s">
         <v>13</v>
       </c>
       <c r="B39" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C39" s="51" t="str">
+      <c r="C39" s="52" t="str">
         <f>B5</f>
-        <v>Javier Ignacio Perez Arenas</v>
-      </c>
-      <c r="D39" s="52"/>
-      <c r="E39" s="52"/>
-      <c r="F39" s="52"/>
-      <c r="G39" s="52"/>
-      <c r="H39" s="52"/>
-      <c r="I39" s="52"/>
-      <c r="J39" s="52"/>
-      <c r="K39" s="53"/>
+        <v>JAVIER IGNACIO PEREZ ARENAS</v>
+      </c>
+      <c r="D39" s="53"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="53"/>
+      <c r="G39" s="53"/>
+      <c r="H39" s="53"/>
+      <c r="I39" s="53"/>
+      <c r="J39" s="53"/>
+      <c r="K39" s="54"/>
     </row>
     <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="62"/>
+      <c r="A40" s="61"/>
       <c r="B40" s="50"/>
-      <c r="C40" s="54"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="55"/>
-      <c r="F40" s="55"/>
-      <c r="G40" s="55"/>
-      <c r="H40" s="55"/>
-      <c r="I40" s="55"/>
-      <c r="J40" s="55"/>
-      <c r="K40" s="56"/>
+      <c r="C40" s="55"/>
+      <c r="D40" s="56"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="56"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="56"/>
+      <c r="J40" s="56"/>
+      <c r="K40" s="57"/>
     </row>
     <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="62"/>
+      <c r="A41" s="61"/>
       <c r="B41" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="57" t="s">
+      <c r="C41" s="51" t="s">
         <v>4</v>
       </c>
       <c r="D41" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E41" s="59"/>
-      <c r="F41" s="59"/>
-      <c r="G41" s="59"/>
-      <c r="H41" s="59"/>
-      <c r="I41" s="59"/>
-      <c r="J41" s="59"/>
-      <c r="K41" s="60"/>
+      <c r="E41" s="62"/>
+      <c r="F41" s="62"/>
+      <c r="G41" s="62"/>
+      <c r="H41" s="62"/>
+      <c r="I41" s="62"/>
+      <c r="J41" s="62"/>
+      <c r="K41" s="59"/>
     </row>
     <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="62"/>
+      <c r="A42" s="61"/>
       <c r="B42" s="15" t="s">
         <v>6</v>
       </c>
@@ -2391,22 +2391,22 @@
       <c r="D42" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E42" s="60"/>
+      <c r="E42" s="59"/>
       <c r="F42" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G42" s="60"/>
+      <c r="G42" s="59"/>
       <c r="H42" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I42" s="60"/>
+      <c r="I42" s="59"/>
       <c r="J42" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K42" s="60"/>
+      <c r="K42" s="59"/>
     </row>
     <row r="43" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="62"/>
+      <c r="A43" s="61"/>
       <c r="B43" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2448,7 +2448,7 @@
       </c>
     </row>
     <row r="44" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A44" s="62"/>
+      <c r="A44" s="61"/>
       <c r="B44" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2490,7 +2490,7 @@
       </c>
     </row>
     <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="62"/>
+      <c r="A45" s="61"/>
       <c r="B45" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2532,7 +2532,7 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="62"/>
+      <c r="A46" s="61"/>
       <c r="B46" s="21" t="s">
         <v>17</v>
       </c>
@@ -2580,59 +2580,59 @@
       <c r="C49" s="23"/>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="61" t="s">
+      <c r="A50" s="60" t="s">
         <v>13</v>
       </c>
       <c r="B50" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C50" s="51" t="str">
+      <c r="C50" s="52" t="str">
         <f>B6</f>
-        <v>Jose Magdiel Gonzalez Lonconanco</v>
-      </c>
-      <c r="D50" s="52"/>
-      <c r="E50" s="52"/>
-      <c r="F50" s="52"/>
-      <c r="G50" s="52"/>
-      <c r="H50" s="52"/>
-      <c r="I50" s="52"/>
-      <c r="J50" s="52"/>
-      <c r="K50" s="53"/>
+        <v>JOSE MAGDIEL GONZALEZ LONCONANCO</v>
+      </c>
+      <c r="D50" s="53"/>
+      <c r="E50" s="53"/>
+      <c r="F50" s="53"/>
+      <c r="G50" s="53"/>
+      <c r="H50" s="53"/>
+      <c r="I50" s="53"/>
+      <c r="J50" s="53"/>
+      <c r="K50" s="54"/>
     </row>
     <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="62"/>
+      <c r="A51" s="61"/>
       <c r="B51" s="50"/>
-      <c r="C51" s="54"/>
-      <c r="D51" s="55"/>
-      <c r="E51" s="55"/>
-      <c r="F51" s="55"/>
-      <c r="G51" s="55"/>
-      <c r="H51" s="55"/>
-      <c r="I51" s="55"/>
-      <c r="J51" s="55"/>
-      <c r="K51" s="56"/>
+      <c r="C51" s="55"/>
+      <c r="D51" s="56"/>
+      <c r="E51" s="56"/>
+      <c r="F51" s="56"/>
+      <c r="G51" s="56"/>
+      <c r="H51" s="56"/>
+      <c r="I51" s="56"/>
+      <c r="J51" s="56"/>
+      <c r="K51" s="57"/>
     </row>
     <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="62"/>
+      <c r="A52" s="61"/>
       <c r="B52" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C52" s="57" t="s">
+      <c r="C52" s="51" t="s">
         <v>4</v>
       </c>
       <c r="D52" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E52" s="59"/>
-      <c r="F52" s="59"/>
-      <c r="G52" s="59"/>
-      <c r="H52" s="59"/>
-      <c r="I52" s="59"/>
-      <c r="J52" s="59"/>
-      <c r="K52" s="60"/>
+      <c r="E52" s="62"/>
+      <c r="F52" s="62"/>
+      <c r="G52" s="62"/>
+      <c r="H52" s="62"/>
+      <c r="I52" s="62"/>
+      <c r="J52" s="62"/>
+      <c r="K52" s="59"/>
     </row>
     <row r="53" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="62"/>
+      <c r="A53" s="61"/>
       <c r="B53" s="15" t="s">
         <v>6</v>
       </c>
@@ -2640,22 +2640,22 @@
       <c r="D53" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E53" s="60"/>
+      <c r="E53" s="59"/>
       <c r="F53" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G53" s="60"/>
+      <c r="G53" s="59"/>
       <c r="H53" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I53" s="60"/>
+      <c r="I53" s="59"/>
       <c r="J53" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K53" s="60"/>
+      <c r="K53" s="59"/>
     </row>
     <row r="54" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="62"/>
+      <c r="A54" s="61"/>
       <c r="B54" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2697,7 +2697,7 @@
       </c>
     </row>
     <row r="55" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A55" s="62"/>
+      <c r="A55" s="61"/>
       <c r="B55" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2739,7 +2739,7 @@
       </c>
     </row>
     <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="62"/>
+      <c r="A56" s="61"/>
       <c r="B56" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2781,7 +2781,7 @@
       </c>
     </row>
     <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="62"/>
+      <c r="A57" s="61"/>
       <c r="B57" s="21" t="s">
         <v>17</v>
       </c>
@@ -3708,17 +3708,14 @@
     <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C50:K51"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="A50:A58"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="D52:K52"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:K40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D41:K41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
     <mergeCell ref="A39:A47"/>
     <mergeCell ref="A27:A35"/>
     <mergeCell ref="E2:E3"/>
@@ -3735,14 +3732,17 @@
     <mergeCell ref="D29:K29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="F30:G30"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:K40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="D41:K41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="D52:K52"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C50:K51"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A50:A58"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:E7">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">

</xml_diff>

<commit_message>
SE AGREGARON LOS PUNTAJES CORRESPONDIENTES
</commit_message>
<xml_diff>
--- a/DOCUMENTOS FASE1/PLANILLA DE EVALUACIÓN FASE 1.xlsx
+++ b/DOCUMENTOS FASE1/PLANILLA DE EVALUACIÓN FASE 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SSDD\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D19073F-846C-4CB4-99A1-B4EE1E99EA5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFDA1BE-F51B-496C-9DC8-03B7B8511C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="100">
   <si>
     <t>INTEGRANTES</t>
   </si>
@@ -393,6 +393,9 @@
   </si>
   <si>
     <t>EMANUEL EDUARDO MEZA BURGOS</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -1059,9 +1062,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1070,15 +1070,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1501,7 +1504,7 @@
       </c>
       <c r="C4" s="6">
         <f>EVALUACION1!$C$24</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4" s="6">
         <f>$C$35</f>
@@ -1509,7 +1512,7 @@
       </c>
       <c r="E4" s="43">
         <f>C4*C$2+D4*D$2</f>
-        <v>7</v>
+        <v>4.75</v>
       </c>
       <c r="G4" s="1"/>
     </row>
@@ -1522,7 +1525,7 @@
       </c>
       <c r="C5" s="6">
         <f>EVALUACION1!$C$24</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5" s="6">
         <f>C47</f>
@@ -1530,7 +1533,7 @@
       </c>
       <c r="E5" s="43">
         <f t="shared" ref="E5:E6" si="0">C5*C$2+D5*D$2</f>
-        <v>7</v>
+        <v>4.75</v>
       </c>
       <c r="G5" s="1"/>
     </row>
@@ -1543,7 +1546,7 @@
       </c>
       <c r="C6" s="6">
         <f>EVALUACION1!$C$24</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D6" s="6">
         <f>C58</f>
@@ -1551,7 +1554,7 @@
       </c>
       <c r="E6" s="43">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>4.75</v>
       </c>
       <c r="G6" s="1"/>
     </row>
@@ -1564,15 +1567,15 @@
       </c>
       <c r="C7" s="6">
         <f>EVALUACION1!$C$24</f>
+        <v>4</v>
+      </c>
+      <c r="D7" s="6">
+        <f>C58</f>
         <v>7</v>
       </c>
-      <c r="D7" s="6">
-        <f>C59</f>
-        <v>0</v>
-      </c>
       <c r="E7" s="43">
-        <f t="shared" ref="E7" si="1">C7*C$2+D7*D$2</f>
-        <v>5.25</v>
+        <f>C7*C$2+D6*D$2</f>
+        <v>4.75</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="18" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -1580,22 +1583,22 @@
         <v>3</v>
       </c>
       <c r="B11" s="14"/>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="57" t="s">
         <v>4</v>
       </c>
       <c r="D11" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62"/>
-      <c r="H11" s="62"/>
-      <c r="I11" s="62"/>
-      <c r="J11" s="62"/>
-      <c r="K11" s="59"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="59"/>
+      <c r="K11" s="60"/>
     </row>
     <row r="12" spans="1:11" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="61"/>
+      <c r="A12" s="62"/>
       <c r="B12" s="24" t="s">
         <v>6</v>
       </c>
@@ -1603,19 +1606,19 @@
       <c r="D12" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="59"/>
+      <c r="E12" s="60"/>
       <c r="F12" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="59"/>
+      <c r="G12" s="60"/>
       <c r="H12" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="I12" s="59"/>
+      <c r="I12" s="60"/>
       <c r="J12" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K12" s="59"/>
+      <c r="K12" s="60"/>
     </row>
     <row r="13" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A13" s="65"/>
@@ -1626,24 +1629,20 @@
       <c r="C13" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="16" t="str">
-        <f t="shared" ref="D13:D16" si="2">IF($C13=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E13" s="16">
+      <c r="D13" s="16"/>
+      <c r="E13" s="16" t="str">
         <f>IF(D13="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F13" s="16" t="str">
-        <f t="shared" ref="F13:F16" si="3">IF($C13=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G13" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G13" s="16">
         <f>IF(F13="X",60*0.1,"")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="H13" s="16" t="str">
-        <f t="shared" ref="H13:H16" si="4">IF($C13=ML,"X","")</f>
+        <f t="shared" ref="H13:H16" si="1">IF($C13=ML,"X","")</f>
         <v/>
       </c>
       <c r="I13" s="16" t="str">
@@ -1651,11 +1650,11 @@
         <v/>
       </c>
       <c r="J13" s="16" t="str">
-        <f t="shared" ref="J13:J16" si="5">IF($C13=NL,"X","")</f>
+        <f t="shared" ref="J13:J16" si="2">IF($C13=NL,"X","")</f>
         <v/>
       </c>
       <c r="K13" s="16" t="str">
-        <f t="shared" ref="K13:K16" si="6">IF($J13="X",0,"")</f>
+        <f t="shared" ref="K13:K16" si="3">IF($J13="X",0,"")</f>
         <v/>
       </c>
     </row>
@@ -1668,40 +1667,36 @@
       <c r="C14" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="16" t="str">
+      <c r="D14" s="16"/>
+      <c r="E14" s="16" t="str">
+        <f t="shared" ref="E14" si="4">IF(D14="X",100*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G14" s="16">
+        <f t="shared" ref="G14" si="5">IF(F14="X",60*0.05,"")</f>
+        <v>3</v>
+      </c>
+      <c r="H14" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I14" s="16" t="str">
+        <f t="shared" ref="I14" si="6">IF(H14="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>X</v>
-      </c>
-      <c r="E14" s="16">
-        <f t="shared" ref="E14" si="7">IF(D14="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F14" s="16" t="str">
+        <v/>
+      </c>
+      <c r="K14" s="16" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="G14" s="16" t="str">
-        <f t="shared" ref="G14" si="8">IF(F14="X",60*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="16" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I14" s="16" t="str">
-        <f t="shared" ref="I14" si="9">IF(H14="X",30*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="16" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K14" s="16" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:11" ht="35.4" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A15" s="65"/>
       <c r="B15" s="35" t="str">
         <f>RUBRICA!A8</f>
@@ -1710,40 +1705,36 @@
       <c r="C15" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="16" t="str">
+      <c r="D15" s="16"/>
+      <c r="E15" s="16" t="str">
+        <f t="shared" ref="E15:E21" si="7">IF(D15="X",100*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G15" s="16">
+        <f t="shared" ref="G15:G21" si="8">IF(F15="X",60*0.05,"")</f>
+        <v>3</v>
+      </c>
+      <c r="H15" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I15" s="16" t="str">
+        <f t="shared" ref="I15:I21" si="9">IF(H15="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>X</v>
-      </c>
-      <c r="E15" s="16">
-        <f t="shared" ref="E15:E21" si="10">IF(D15="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F15" s="16" t="str">
+        <v/>
+      </c>
+      <c r="K15" s="16" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="G15" s="16" t="str">
-        <f t="shared" ref="G15:G21" si="11">IF(F15="X",60*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="H15" s="16" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I15" s="16" t="str">
-        <f t="shared" ref="I15:I21" si="12">IF(H15="X",30*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="16" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K15" s="16" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:11" ht="34.200000000000003" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A16" s="65"/>
       <c r="B16" s="35" t="str">
         <f>RUBRICA!A9</f>
@@ -1752,24 +1743,20 @@
       <c r="C16" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="16" t="str">
-        <f t="shared" si="2"/>
-        <v>X</v>
-      </c>
-      <c r="E16" s="16">
+      <c r="D16" s="16"/>
+      <c r="E16" s="16" t="str">
         <f>IF(D16="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F16" s="16" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G16" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G16" s="16">
         <f>IF(F16="X",60*0.05,"")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="H16" s="16" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="I16" s="16" t="str">
@@ -1777,11 +1764,11 @@
         <v/>
       </c>
       <c r="J16" s="16" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="K16" s="16" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -1794,36 +1781,32 @@
       <c r="C17" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="16" t="str">
-        <f t="shared" ref="D17:D22" si="13">IF($C17=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E17" s="16">
-        <f t="shared" ref="E17" si="14">IF(D17="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F17" s="16" t="str">
-        <f t="shared" ref="F17:F22" si="15">IF($C17=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G17" s="16" t="str">
-        <f t="shared" ref="G17" si="16">IF(F17="X",60*0.1,"")</f>
-        <v/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16" t="str">
+        <f t="shared" ref="E17" si="10">IF(D17="X",100*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" s="16">
+        <f t="shared" ref="G17" si="11">IF(F17="X",60*0.1,"")</f>
+        <v>6</v>
       </c>
       <c r="H17" s="16" t="str">
-        <f t="shared" ref="H17:H22" si="17">IF($C17=ML,"X","")</f>
+        <f t="shared" ref="H17:H22" si="12">IF($C17=ML,"X","")</f>
         <v/>
       </c>
       <c r="I17" s="16" t="str">
-        <f t="shared" ref="I17" si="18">IF(H17="X",30*0.1,"")</f>
+        <f t="shared" ref="I17" si="13">IF(H17="X",30*0.1,"")</f>
         <v/>
       </c>
       <c r="J17" s="16" t="str">
-        <f t="shared" ref="J17:J22" si="19">IF($C17=NL,"X","")</f>
+        <f t="shared" ref="J17:J22" si="14">IF($C17=NL,"X","")</f>
         <v/>
       </c>
       <c r="K17" s="16" t="str">
-        <f t="shared" ref="K17:K22" si="20">IF($J17="X",0,"")</f>
+        <f t="shared" ref="K17:K22" si="15">IF($J17="X",0,"")</f>
         <v/>
       </c>
     </row>
@@ -1836,36 +1819,32 @@
       <c r="C18" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="16" t="str">
-        <f t="shared" si="13"/>
-        <v>X</v>
-      </c>
-      <c r="E18" s="16">
-        <f t="shared" ref="E18" si="21">IF(D18="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F18" s="16" t="str">
+      <c r="D18" s="16"/>
+      <c r="E18" s="16" t="str">
+        <f t="shared" ref="E18" si="16">IF(D18="X",100*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G18" s="16">
+        <f t="shared" ref="G18" si="17">IF(F18="X",60*0.1,"")</f>
+        <v>6</v>
+      </c>
+      <c r="H18" s="16" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="I18" s="16" t="str">
+        <f t="shared" ref="I18" si="18">IF(H18="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="K18" s="16" t="str">
         <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="G18" s="16" t="str">
-        <f t="shared" ref="G18" si="22">IF(F18="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H18" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="I18" s="16" t="str">
-        <f t="shared" ref="I18" si="23">IF(H18="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J18" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="K18" s="16" t="str">
-        <f t="shared" si="20"/>
         <v/>
       </c>
     </row>
@@ -1878,36 +1857,32 @@
       <c r="C19" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="16" t="str">
-        <f t="shared" si="13"/>
-        <v>X</v>
-      </c>
-      <c r="E19" s="16">
+      <c r="D19" s="16"/>
+      <c r="E19" s="16" t="str">
         <f>IF(D19="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F19" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F19" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G19" s="16">
+        <f t="shared" ref="G19" si="19">IF(F19="X",60*0.05,"")</f>
+        <v>3</v>
+      </c>
+      <c r="H19" s="16" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="I19" s="16" t="str">
+        <f t="shared" ref="I19" si="20">IF(H19="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="K19" s="16" t="str">
         <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="G19" s="16" t="str">
-        <f t="shared" ref="G19" si="24">IF(F19="X",60*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="H19" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="I19" s="16" t="str">
-        <f t="shared" ref="I19" si="25">IF(H19="X",30*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="K19" s="16" t="str">
-        <f t="shared" si="20"/>
         <v/>
       </c>
     </row>
@@ -1920,36 +1895,32 @@
       <c r="C20" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="16" t="str">
-        <f t="shared" si="13"/>
-        <v>X</v>
-      </c>
-      <c r="E20" s="16">
+      <c r="D20" s="16"/>
+      <c r="E20" s="16" t="str">
         <f>IF(D20="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F20" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G20" s="16">
+        <f t="shared" si="8"/>
+        <v>3</v>
+      </c>
+      <c r="H20" s="16" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="I20" s="16" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="J20" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="K20" s="16" t="str">
         <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="G20" s="16" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="H20" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="I20" s="16" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="J20" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="K20" s="16" t="str">
-        <f t="shared" si="20"/>
         <v/>
       </c>
     </row>
@@ -1962,36 +1933,32 @@
       <c r="C21" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D21" s="16" t="str">
-        <f t="shared" si="13"/>
-        <v>X</v>
-      </c>
-      <c r="E21" s="16">
-        <f t="shared" si="10"/>
-        <v>5</v>
-      </c>
-      <c r="F21" s="16" t="str">
+      <c r="D21" s="16"/>
+      <c r="E21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G21" s="16">
+        <f t="shared" si="8"/>
+        <v>3</v>
+      </c>
+      <c r="H21" s="16" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="I21" s="16" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="J21" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="K21" s="16" t="str">
         <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="G21" s="16" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="H21" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="I21" s="16" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="J21" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="K21" s="16" t="str">
-        <f t="shared" si="20"/>
         <v/>
       </c>
     </row>
@@ -2005,24 +1972,20 @@
       <c r="C22" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D22" s="16" t="str">
-        <f t="shared" si="13"/>
-        <v>X</v>
-      </c>
-      <c r="E22" s="16">
+      <c r="D22" s="16"/>
+      <c r="E22" s="16" t="str">
         <f>IF(D22="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F22" s="16" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="G22" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G22" s="16">
         <f>IF(F22="X",60*0.1,"")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="H22" s="16" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="I22" s="16" t="str">
@@ -2030,32 +1993,32 @@
         <v/>
       </c>
       <c r="J22" s="16" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="K22" s="16" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="61"/>
+      <c r="A23" s="62"/>
       <c r="B23" s="34" t="s">
         <v>11</v>
       </c>
       <c r="C23" s="37">
         <f>E23+G23+I23+K23</f>
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="D23" s="19"/>
       <c r="E23" s="19">
         <f>SUM(E13:E22)</f>
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F23" s="19"/>
       <c r="G23" s="19">
         <f>SUM(G13:G22)</f>
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="H23" s="19"/>
       <c r="I23" s="19">
@@ -2075,65 +2038,65 @@
       </c>
       <c r="C24" s="20">
         <f>VLOOKUP(C23,ESCALA_IEP!A2:B142,2,FALSE)</f>
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="60" t="s">
+      <c r="A27" s="61" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="52" t="str">
+      <c r="C27" s="51" t="str">
         <f>$B$4</f>
         <v>RAUL IGNACIO IBARRA CARVAJAL</v>
       </c>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="53"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="53"/>
-      <c r="I27" s="53"/>
-      <c r="J27" s="53"/>
-      <c r="K27" s="54"/>
+      <c r="D27" s="52"/>
+      <c r="E27" s="52"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="52"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="52"/>
+      <c r="J27" s="52"/>
+      <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="61"/>
+      <c r="A28" s="62"/>
       <c r="B28" s="50"/>
-      <c r="C28" s="55"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="56"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
-      <c r="I28" s="56"/>
-      <c r="J28" s="56"/>
-      <c r="K28" s="57"/>
+      <c r="C28" s="54"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="55"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="55"/>
+      <c r="I28" s="55"/>
+      <c r="J28" s="55"/>
+      <c r="K28" s="56"/>
     </row>
     <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="61"/>
+      <c r="A29" s="62"/>
       <c r="B29" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="51" t="s">
+      <c r="C29" s="57" t="s">
         <v>4</v>
       </c>
       <c r="D29" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E29" s="62"/>
-      <c r="F29" s="62"/>
-      <c r="G29" s="62"/>
-      <c r="H29" s="62"/>
-      <c r="I29" s="62"/>
-      <c r="J29" s="62"/>
-      <c r="K29" s="59"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="59"/>
+      <c r="G29" s="59"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="59"/>
+      <c r="K29" s="60"/>
     </row>
     <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="61"/>
+      <c r="A30" s="62"/>
       <c r="B30" s="15" t="s">
         <v>6</v>
       </c>
@@ -2141,22 +2104,22 @@
       <c r="D30" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="59"/>
+      <c r="E30" s="60"/>
       <c r="F30" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G30" s="59"/>
+      <c r="G30" s="60"/>
       <c r="H30" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I30" s="59"/>
+      <c r="I30" s="60"/>
       <c r="J30" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K30" s="59"/>
+      <c r="K30" s="60"/>
     </row>
     <row r="31" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="61"/>
+      <c r="A31" s="62"/>
       <c r="B31" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2164,24 +2127,20 @@
       <c r="C31" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="16" t="str">
-        <f t="shared" ref="D31:D32" si="26">IF($C31=CL,"X","")</f>
-        <v>X</v>
+      <c r="D31" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E31" s="16">
         <f>IF(D31="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F31" s="16" t="str">
-        <f t="shared" ref="F31:F32" si="27">IF($C31=L,"X","")</f>
-        <v/>
-      </c>
+      <c r="F31" s="16"/>
       <c r="G31" s="16" t="str">
         <f>IF(F31="X",60*0.1,"")</f>
         <v/>
       </c>
       <c r="H31" s="16" t="str">
-        <f t="shared" ref="H31:H32" si="28">IF($C31=ML,"X","")</f>
+        <f t="shared" ref="H31:H32" si="21">IF($C31=ML,"X","")</f>
         <v/>
       </c>
       <c r="I31" s="16" t="str">
@@ -2189,16 +2148,16 @@
         <v/>
       </c>
       <c r="J31" s="16" t="str">
-        <f t="shared" ref="J31:J32" si="29">IF($C31=NL,"X","")</f>
+        <f t="shared" ref="J31:J32" si="22">IF($C31=NL,"X","")</f>
         <v/>
       </c>
       <c r="K31" s="16" t="str">
-        <f t="shared" ref="K31:K32" si="30">IF($J31="X",0,"")</f>
+        <f t="shared" ref="K31:K32" si="23">IF($J31="X",0,"")</f>
         <v/>
       </c>
     </row>
     <row r="32" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="61"/>
+      <c r="A32" s="62"/>
       <c r="B32" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2206,24 +2165,20 @@
       <c r="C32" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D32" s="16" t="str">
-        <f t="shared" si="26"/>
-        <v>X</v>
+      <c r="D32" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E32" s="16">
         <f>IF(D32="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F32" s="16" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
+      <c r="F32" s="16"/>
       <c r="G32" s="16" t="str">
         <f>IF(F32="X",60*0.1,"")</f>
         <v/>
       </c>
       <c r="H32" s="16" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="I32" s="16" t="str">
@@ -2231,16 +2186,16 @@
         <v/>
       </c>
       <c r="J32" s="16" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
       <c r="K32" s="16" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
     <row r="33" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="61"/>
+      <c r="A33" s="62"/>
       <c r="B33" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2248,18 +2203,14 @@
       <c r="C33" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D33" s="16" t="str">
-        <f>IF($C33=CL,"X","")</f>
-        <v>X</v>
+      <c r="D33" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E33" s="16">
         <f>IF(D33="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F33" s="16" t="str">
-        <f>IF($C33=L,"X","")</f>
-        <v/>
-      </c>
+      <c r="F33" s="16"/>
       <c r="G33" s="16" t="str">
         <f>IF(F33="X",60*0.1,"")</f>
         <v/>
@@ -2282,7 +2233,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="61"/>
+      <c r="A34" s="62"/>
       <c r="B34" s="21" t="s">
         <v>17</v>
       </c>
@@ -2297,17 +2248,17 @@
       </c>
       <c r="F34" s="19"/>
       <c r="G34" s="19">
-        <f t="shared" ref="G34:K34" si="31">SUM(G31:G33)</f>
+        <f t="shared" ref="G34:K34" si="24">SUM(G31:G33)</f>
         <v>0</v>
       </c>
       <c r="H34" s="19"/>
       <c r="I34" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="J34" s="19"/>
       <c r="K34" s="19">
-        <f t="shared" si="31"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -2331,59 +2282,59 @@
     </row>
     <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="60" t="s">
+      <c r="A39" s="61" t="s">
         <v>13</v>
       </c>
       <c r="B39" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C39" s="52" t="str">
+      <c r="C39" s="51" t="str">
         <f>B5</f>
         <v>JAVIER IGNACIO PEREZ ARENAS</v>
       </c>
-      <c r="D39" s="53"/>
-      <c r="E39" s="53"/>
-      <c r="F39" s="53"/>
-      <c r="G39" s="53"/>
-      <c r="H39" s="53"/>
-      <c r="I39" s="53"/>
-      <c r="J39" s="53"/>
-      <c r="K39" s="54"/>
+      <c r="D39" s="52"/>
+      <c r="E39" s="52"/>
+      <c r="F39" s="52"/>
+      <c r="G39" s="52"/>
+      <c r="H39" s="52"/>
+      <c r="I39" s="52"/>
+      <c r="J39" s="52"/>
+      <c r="K39" s="53"/>
     </row>
     <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="61"/>
+      <c r="A40" s="62"/>
       <c r="B40" s="50"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="56"/>
-      <c r="E40" s="56"/>
-      <c r="F40" s="56"/>
-      <c r="G40" s="56"/>
-      <c r="H40" s="56"/>
-      <c r="I40" s="56"/>
-      <c r="J40" s="56"/>
-      <c r="K40" s="57"/>
+      <c r="C40" s="54"/>
+      <c r="D40" s="55"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="55"/>
+      <c r="H40" s="55"/>
+      <c r="I40" s="55"/>
+      <c r="J40" s="55"/>
+      <c r="K40" s="56"/>
     </row>
     <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="61"/>
+      <c r="A41" s="62"/>
       <c r="B41" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="51" t="s">
+      <c r="C41" s="57" t="s">
         <v>4</v>
       </c>
       <c r="D41" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E41" s="62"/>
-      <c r="F41" s="62"/>
-      <c r="G41" s="62"/>
-      <c r="H41" s="62"/>
-      <c r="I41" s="62"/>
-      <c r="J41" s="62"/>
-      <c r="K41" s="59"/>
+      <c r="E41" s="59"/>
+      <c r="F41" s="59"/>
+      <c r="G41" s="59"/>
+      <c r="H41" s="59"/>
+      <c r="I41" s="59"/>
+      <c r="J41" s="59"/>
+      <c r="K41" s="60"/>
     </row>
     <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="61"/>
+      <c r="A42" s="62"/>
       <c r="B42" s="15" t="s">
         <v>6</v>
       </c>
@@ -2391,22 +2342,22 @@
       <c r="D42" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E42" s="59"/>
+      <c r="E42" s="60"/>
       <c r="F42" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G42" s="59"/>
+      <c r="G42" s="60"/>
       <c r="H42" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I42" s="59"/>
+      <c r="I42" s="60"/>
       <c r="J42" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K42" s="59"/>
+      <c r="K42" s="60"/>
     </row>
     <row r="43" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="61"/>
+      <c r="A43" s="62"/>
       <c r="B43" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2414,24 +2365,20 @@
       <c r="C43" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D43" s="16" t="str">
-        <f t="shared" ref="D43:D44" si="32">IF($C43=CL,"X","")</f>
-        <v>X</v>
+      <c r="D43" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E43" s="16">
         <f>IF(D43="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F43" s="16" t="str">
-        <f t="shared" ref="F43:F44" si="33">IF($C43=L,"X","")</f>
-        <v/>
-      </c>
+      <c r="F43" s="16"/>
       <c r="G43" s="16" t="str">
         <f>IF(F43="X",60*0.1,"")</f>
         <v/>
       </c>
       <c r="H43" s="16" t="str">
-        <f t="shared" ref="H43:H44" si="34">IF($C43=ML,"X","")</f>
+        <f t="shared" ref="H43:H44" si="25">IF($C43=ML,"X","")</f>
         <v/>
       </c>
       <c r="I43" s="16" t="str">
@@ -2439,16 +2386,16 @@
         <v/>
       </c>
       <c r="J43" s="16" t="str">
-        <f t="shared" ref="J43:J44" si="35">IF($C43=NL,"X","")</f>
+        <f t="shared" ref="J43:J44" si="26">IF($C43=NL,"X","")</f>
         <v/>
       </c>
       <c r="K43" s="16" t="str">
-        <f t="shared" ref="K43:K44" si="36">IF($J43="X",0,"")</f>
+        <f t="shared" ref="K43:K44" si="27">IF($J43="X",0,"")</f>
         <v/>
       </c>
     </row>
     <row r="44" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A44" s="61"/>
+      <c r="A44" s="62"/>
       <c r="B44" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2456,24 +2403,20 @@
       <c r="C44" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D44" s="16" t="str">
-        <f t="shared" si="32"/>
-        <v>X</v>
+      <c r="D44" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E44" s="16">
         <f>IF(D44="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F44" s="16" t="str">
-        <f t="shared" si="33"/>
-        <v/>
-      </c>
+      <c r="F44" s="16"/>
       <c r="G44" s="16" t="str">
         <f>IF(F44="X",60*0.1,"")</f>
         <v/>
       </c>
       <c r="H44" s="16" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
       <c r="I44" s="16" t="str">
@@ -2481,16 +2424,16 @@
         <v/>
       </c>
       <c r="J44" s="16" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
       <c r="K44" s="16" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
     </row>
     <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="61"/>
+      <c r="A45" s="62"/>
       <c r="B45" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2498,18 +2441,14 @@
       <c r="C45" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D45" s="16" t="str">
-        <f>IF($C45=CL,"X","")</f>
-        <v>X</v>
+      <c r="D45" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E45" s="16">
         <f>IF(D45="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F45" s="16" t="str">
-        <f>IF($C45=L,"X","")</f>
-        <v/>
-      </c>
+      <c r="F45" s="16"/>
       <c r="G45" s="16" t="str">
         <f>IF(F45="X",60*0.1,"")</f>
         <v/>
@@ -2532,7 +2471,7 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="61"/>
+      <c r="A46" s="62"/>
       <c r="B46" s="21" t="s">
         <v>17</v>
       </c>
@@ -2547,17 +2486,17 @@
       </c>
       <c r="F46" s="19"/>
       <c r="G46" s="19">
-        <f t="shared" ref="G46" si="37">SUM(G43:G45)</f>
+        <f t="shared" ref="G46" si="28">SUM(G43:G45)</f>
         <v>0</v>
       </c>
       <c r="H46" s="19"/>
       <c r="I46" s="19">
-        <f t="shared" ref="I46" si="38">SUM(I43:I45)</f>
+        <f t="shared" ref="I46" si="29">SUM(I43:I45)</f>
         <v>0</v>
       </c>
       <c r="J46" s="19"/>
       <c r="K46" s="19">
-        <f t="shared" ref="K46" si="39">SUM(K43:K45)</f>
+        <f t="shared" ref="K46" si="30">SUM(K43:K45)</f>
         <v>0</v>
       </c>
     </row>
@@ -2580,59 +2519,59 @@
       <c r="C49" s="23"/>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="60" t="s">
+      <c r="A50" s="61" t="s">
         <v>13</v>
       </c>
       <c r="B50" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C50" s="52" t="str">
+      <c r="C50" s="51" t="str">
         <f>B6</f>
         <v>JOSE MAGDIEL GONZALEZ LONCONANCO</v>
       </c>
-      <c r="D50" s="53"/>
-      <c r="E50" s="53"/>
-      <c r="F50" s="53"/>
-      <c r="G50" s="53"/>
-      <c r="H50" s="53"/>
-      <c r="I50" s="53"/>
-      <c r="J50" s="53"/>
-      <c r="K50" s="54"/>
+      <c r="D50" s="52"/>
+      <c r="E50" s="52"/>
+      <c r="F50" s="52"/>
+      <c r="G50" s="52"/>
+      <c r="H50" s="52"/>
+      <c r="I50" s="52"/>
+      <c r="J50" s="52"/>
+      <c r="K50" s="53"/>
     </row>
     <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="61"/>
+      <c r="A51" s="62"/>
       <c r="B51" s="50"/>
-      <c r="C51" s="55"/>
-      <c r="D51" s="56"/>
-      <c r="E51" s="56"/>
-      <c r="F51" s="56"/>
-      <c r="G51" s="56"/>
-      <c r="H51" s="56"/>
-      <c r="I51" s="56"/>
-      <c r="J51" s="56"/>
-      <c r="K51" s="57"/>
+      <c r="C51" s="54"/>
+      <c r="D51" s="55"/>
+      <c r="E51" s="55"/>
+      <c r="F51" s="55"/>
+      <c r="G51" s="55"/>
+      <c r="H51" s="55"/>
+      <c r="I51" s="55"/>
+      <c r="J51" s="55"/>
+      <c r="K51" s="56"/>
     </row>
     <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="61"/>
+      <c r="A52" s="62"/>
       <c r="B52" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C52" s="51" t="s">
+      <c r="C52" s="57" t="s">
         <v>4</v>
       </c>
       <c r="D52" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E52" s="62"/>
-      <c r="F52" s="62"/>
-      <c r="G52" s="62"/>
-      <c r="H52" s="62"/>
-      <c r="I52" s="62"/>
-      <c r="J52" s="62"/>
-      <c r="K52" s="59"/>
+      <c r="E52" s="59"/>
+      <c r="F52" s="59"/>
+      <c r="G52" s="59"/>
+      <c r="H52" s="59"/>
+      <c r="I52" s="59"/>
+      <c r="J52" s="59"/>
+      <c r="K52" s="60"/>
     </row>
     <row r="53" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="61"/>
+      <c r="A53" s="62"/>
       <c r="B53" s="15" t="s">
         <v>6</v>
       </c>
@@ -2640,22 +2579,22 @@
       <c r="D53" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E53" s="59"/>
+      <c r="E53" s="60"/>
       <c r="F53" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G53" s="59"/>
+      <c r="G53" s="60"/>
       <c r="H53" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I53" s="59"/>
+      <c r="I53" s="60"/>
       <c r="J53" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K53" s="59"/>
+      <c r="K53" s="60"/>
     </row>
     <row r="54" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="61"/>
+      <c r="A54" s="62"/>
       <c r="B54" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2663,24 +2602,20 @@
       <c r="C54" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D54" s="16" t="str">
-        <f t="shared" ref="D54:D55" si="40">IF($C54=CL,"X","")</f>
-        <v>X</v>
+      <c r="D54" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E54" s="16">
         <f>IF(D54="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F54" s="16" t="str">
-        <f t="shared" ref="F54:F55" si="41">IF($C54=L,"X","")</f>
-        <v/>
-      </c>
+      <c r="F54" s="16"/>
       <c r="G54" s="16" t="str">
         <f>IF(F54="X",60*0.1,"")</f>
         <v/>
       </c>
       <c r="H54" s="16" t="str">
-        <f t="shared" ref="H54:H55" si="42">IF($C54=ML,"X","")</f>
+        <f t="shared" ref="H54:H55" si="31">IF($C54=ML,"X","")</f>
         <v/>
       </c>
       <c r="I54" s="16" t="str">
@@ -2688,16 +2623,16 @@
         <v/>
       </c>
       <c r="J54" s="16" t="str">
-        <f t="shared" ref="J54:J55" si="43">IF($C54=NL,"X","")</f>
+        <f t="shared" ref="J54:J55" si="32">IF($C54=NL,"X","")</f>
         <v/>
       </c>
       <c r="K54" s="16" t="str">
-        <f t="shared" ref="K54:K55" si="44">IF($J54="X",0,"")</f>
+        <f t="shared" ref="K54:K55" si="33">IF($J54="X",0,"")</f>
         <v/>
       </c>
     </row>
     <row r="55" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A55" s="61"/>
+      <c r="A55" s="62"/>
       <c r="B55" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2705,24 +2640,20 @@
       <c r="C55" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D55" s="16" t="str">
-        <f t="shared" si="40"/>
-        <v>X</v>
+      <c r="D55" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E55" s="16">
         <f>IF(D55="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F55" s="16" t="str">
-        <f t="shared" si="41"/>
-        <v/>
-      </c>
+      <c r="F55" s="16"/>
       <c r="G55" s="16" t="str">
         <f>IF(F55="X",60*0.1,"")</f>
         <v/>
       </c>
       <c r="H55" s="16" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="I55" s="16" t="str">
@@ -2730,16 +2661,16 @@
         <v/>
       </c>
       <c r="J55" s="16" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
       <c r="K55" s="16" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
     </row>
     <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="61"/>
+      <c r="A56" s="62"/>
       <c r="B56" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2747,18 +2678,14 @@
       <c r="C56" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D56" s="16" t="str">
-        <f>IF($C56=CL,"X","")</f>
-        <v>X</v>
+      <c r="D56" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="E56" s="16">
         <f>IF(D56="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F56" s="16" t="str">
-        <f>IF($C56=L,"X","")</f>
-        <v/>
-      </c>
+      <c r="F56" s="16"/>
       <c r="G56" s="16" t="str">
         <f>IF(F56="X",60*0.1,"")</f>
         <v/>
@@ -2781,7 +2708,7 @@
       </c>
     </row>
     <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="61"/>
+      <c r="A57" s="62"/>
       <c r="B57" s="21" t="s">
         <v>17</v>
       </c>
@@ -2798,27 +2725,27 @@
         <v>30</v>
       </c>
       <c r="F57" s="19">
-        <f t="shared" ref="F57" si="45">SUM(F54:F56)</f>
+        <f t="shared" ref="F57" si="34">SUM(F54:F56)</f>
         <v>0</v>
       </c>
       <c r="G57" s="19">
-        <f t="shared" ref="G57" si="46">SUM(G54:G56)</f>
+        <f t="shared" ref="G57" si="35">SUM(G54:G56)</f>
         <v>0</v>
       </c>
       <c r="H57" s="19">
-        <f t="shared" ref="H57" si="47">SUM(H54:H56)</f>
+        <f t="shared" ref="H57" si="36">SUM(H54:H56)</f>
         <v>0</v>
       </c>
       <c r="I57" s="19">
-        <f t="shared" ref="I57" si="48">SUM(I54:I56)</f>
+        <f t="shared" ref="I57" si="37">SUM(I54:I56)</f>
         <v>0</v>
       </c>
       <c r="J57" s="19">
-        <f t="shared" ref="J57" si="49">SUM(J54:J56)</f>
+        <f t="shared" ref="J57" si="38">SUM(J54:J56)</f>
         <v>0</v>
       </c>
       <c r="K57" s="19">
-        <f t="shared" ref="K57" si="50">SUM(K54:K56)</f>
+        <f t="shared" ref="K57" si="39">SUM(K54:K56)</f>
         <v>0</v>
       </c>
     </row>
@@ -2837,26 +2764,258 @@
       <c r="C59" s="23"/>
     </row>
     <row r="60" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="61" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" s="51" t="str">
+        <f>B7</f>
+        <v>EMANUEL EDUARDO MEZA BURGOS</v>
+      </c>
+      <c r="D61" s="52"/>
+      <c r="E61" s="52"/>
+      <c r="F61" s="52"/>
+      <c r="G61" s="52"/>
+      <c r="H61" s="52"/>
+      <c r="I61" s="52"/>
+      <c r="J61" s="52"/>
+      <c r="K61" s="53"/>
+    </row>
+    <row r="62" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="62"/>
+      <c r="B62" s="50"/>
+      <c r="C62" s="54"/>
+      <c r="D62" s="55"/>
+      <c r="E62" s="55"/>
+      <c r="F62" s="55"/>
+      <c r="G62" s="55"/>
+      <c r="H62" s="55"/>
+      <c r="I62" s="55"/>
+      <c r="J62" s="55"/>
+      <c r="K62" s="56"/>
+    </row>
+    <row r="63" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="62"/>
+      <c r="B63" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C63" s="57" t="s">
+        <v>4</v>
+      </c>
+      <c r="D63" s="58" t="s">
+        <v>5</v>
+      </c>
+      <c r="E63" s="59"/>
+      <c r="F63" s="59"/>
+      <c r="G63" s="59"/>
+      <c r="H63" s="59"/>
+      <c r="I63" s="59"/>
+      <c r="J63" s="59"/>
+      <c r="K63" s="60"/>
+    </row>
+    <row r="64" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="62"/>
+      <c r="B64" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C64" s="50"/>
+      <c r="D64" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="E64" s="60"/>
+      <c r="F64" s="58" t="s">
+        <v>8</v>
+      </c>
+      <c r="G64" s="60"/>
+      <c r="H64" s="58" t="s">
+        <v>16</v>
+      </c>
+      <c r="I64" s="60"/>
+      <c r="J64" s="58" t="s">
+        <v>10</v>
+      </c>
+      <c r="K64" s="60"/>
+    </row>
+    <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="62"/>
+      <c r="B65" s="35" t="str">
+        <f>RUBRICA!A7</f>
+        <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
+      </c>
+      <c r="C65" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E65" s="16">
+        <f>IF(D65="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F65" s="16"/>
+      <c r="G65" s="16" t="str">
+        <f>IF(F65="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H65" s="16" t="str">
+        <f t="shared" ref="H65:H66" si="40">IF($C65=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I65" s="16" t="str">
+        <f>IF(H65="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J65" s="16" t="str">
+        <f t="shared" ref="J65:J66" si="41">IF($C65=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K65" s="16" t="str">
+        <f t="shared" ref="K65:K66" si="42">IF($J65="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="62"/>
+      <c r="B66" s="35" t="str">
+        <f>RUBRICA!A15</f>
+        <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
+      </c>
+      <c r="C66" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E66" s="16">
+        <f>IF(D66="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F66" s="16"/>
+      <c r="G66" s="16" t="str">
+        <f>IF(F66="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H66" s="16" t="str">
+        <f t="shared" si="40"/>
+        <v/>
+      </c>
+      <c r="I66" s="16" t="str">
+        <f>IF(H66="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J66" s="16" t="str">
+        <f t="shared" si="41"/>
+        <v/>
+      </c>
+      <c r="K66" s="16" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="62"/>
+      <c r="B67" s="35" t="str">
+        <f>RUBRICA!A17</f>
+        <v>13. Colaboración y trabajo en equipo *</v>
+      </c>
+      <c r="C67" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E67" s="16">
+        <f>IF(D67="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F67" s="16"/>
+      <c r="G67" s="16" t="str">
+        <f>IF(F67="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H67" s="16" t="str">
+        <f>IF($C67=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I67" s="16" t="str">
+        <f>IF(H67="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J67" s="16" t="str">
+        <f>IF($C67=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K67" s="16" t="str">
+        <f>IF($J67="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="62"/>
+      <c r="B68" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C68" s="18">
+        <f>E68+G68+I68+K68</f>
+        <v>30</v>
+      </c>
+      <c r="D68" s="19">
+        <f>COUNTIF(D66:D67,"X")</f>
+        <v>2</v>
+      </c>
+      <c r="E68" s="19">
+        <f>SUM(E65:E67)</f>
+        <v>30</v>
+      </c>
+      <c r="F68" s="19">
+        <f t="shared" ref="F68:K68" si="43">SUM(F65:F67)</f>
+        <v>0</v>
+      </c>
+      <c r="G68" s="19">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="H68" s="19">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="I68" s="19">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="J68" s="19">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="K68" s="19">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="50"/>
+      <c r="B69" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C69" s="20">
+        <f>VLOOKUP(C57,ESCALA_TRAB_EQUIP!A2:B62,2,FALSE)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="71" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="72" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="73" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="74" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="75" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="76" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="77" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="79" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="80" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -3707,15 +3866,27 @@
     <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:K40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="D41:K41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
+  <mergeCells count="44">
+    <mergeCell ref="A61:A69"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="C61:K62"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="D63:K63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="H64:I64"/>
+    <mergeCell ref="J64:K64"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C50:K51"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A50:A58"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="D52:K52"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="H53:I53"/>
     <mergeCell ref="A39:A47"/>
     <mergeCell ref="A27:A35"/>
     <mergeCell ref="E2:E3"/>
@@ -3732,17 +3903,14 @@
     <mergeCell ref="D29:K29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="D52:K52"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C50:K51"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="A50:A58"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:K40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D41:K41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:E7">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
@@ -3767,7 +3935,7 @@
           <x14:formula1>
             <xm:f>'RELEVANCIA-PUNTAJE'!$B$2:$E$2</xm:f>
           </x14:formula1>
-          <xm:sqref>C13:C22 C54:C56 C43:C45 C31:C33</xm:sqref>
+          <xm:sqref>C13:C22 C54:C56 C43:C45 C31:C33 C65:C67</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>